<commit_message>
feat(crm): world-class loyalty CRM — members, points, rewards, gamification, referrals, member app (OTP+LINE), spin-the-wheel, campaigns, partner privileges, analytics, SoD R14–R16 (#69)
Complete Buzzebees-class, audit-grade loyalty CRM (P1–P4). Points-as-liability GL (TFRS 15, acct 2250); rewards/coupons; tiers/missions; referrals; phone-OTP + LINE member app (/m); spin-the-wheel; segmented/scheduled campaigns; formal crm_* permissions + SoD R14–R16; partner privileges; churn/redemption analytics. 13 ICFR control checks (LYL-03..16), 25 UAT cases, all docs synced. Six adversarial reviews; three caught real defects (OTP cap, campaign re-fire, unjournaled migrations) — all fixed and harness-locked. Verified: 75/75 CI checks.
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SoD_Matrix_v1.xlsx
+++ b/compliance/Oshinei_ERP_SoD_Matrix_v1.xlsx
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Permission Inventory'!$A$1:$F$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SoD Rules'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SoD Rules'!$A$1:$H$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Detected Conflicts'!$A$1:$H$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -762,7 +762,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>13 SoD conflict rules; a role conflicts when it holds duties on BOTH sides of a rule</t>
+          <t>16 SoD conflict rules; a role conflicts when it holds duties on BOTH sides of a rule</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2718,8 +2718,134 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Configure rewards / vouchers</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>POS redemption at till</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>crm_reward</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>pos_sell</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Create a reward/voucher and redeem it for oneself at the till.</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Separate reward-catalog configuration from POS redemption; review reward-change + redemption reports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Manual points adjustment</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Member master maintenance</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>crm_points_adjust</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>crm_member</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Enrol a ghost member and credit points to it.</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Separate member enrolment from points adjustment; over-threshold adjust via maker-checker approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Campaign issuance of point-bearing value</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Points adjustment</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>crm_campaign</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>crm_points_adjust</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Self-issue loyalty value through two channels (campaign coupons + manual adjustment).</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Separate campaign issuance from points adjustment; review issuance + adjustment logs.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3847,7 +3973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3864,7 +3990,10 @@
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="6" customWidth="1" min="13" max="13"/>
     <col width="6" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -3940,6 +4069,21 @@
       </c>
       <c r="O1" s="21" t="inlineStr">
         <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="P1" s="21" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="Q1" s="21" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="R1" s="21" t="inlineStr">
+        <is>
           <t># Conflicts</t>
         </is>
       </c>
@@ -4015,7 +4159,22 @@
           <t>▲</t>
         </is>
       </c>
-      <c r="O2" s="24" t="inlineStr">
+      <c r="O2" s="23" t="inlineStr">
+        <is>
+          <t>▲</t>
+        </is>
+      </c>
+      <c r="P2" s="23" t="inlineStr">
+        <is>
+          <t>▲</t>
+        </is>
+      </c>
+      <c r="Q2" s="23" t="inlineStr">
+        <is>
+          <t>▲</t>
+        </is>
+      </c>
+      <c r="R2" s="24" t="inlineStr">
         <is>
           <t>ALL (▲)</t>
         </is>
@@ -4092,7 +4251,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O3" s="20" t="n">
+      <c r="O3" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P3" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q3" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R3" s="20" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4167,7 +4341,22 @@
           <t>✕</t>
         </is>
       </c>
-      <c r="O4" s="20" t="n">
+      <c r="O4" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P4" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q4" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R4" s="20" t="n">
         <v>4</v>
       </c>
     </row>
@@ -4242,7 +4431,22 @@
           <t>✕</t>
         </is>
       </c>
-      <c r="O5" s="20" t="n">
+      <c r="O5" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P5" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q5" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R5" s="20" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4317,7 +4521,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O6" s="20" t="n">
+      <c r="O6" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P6" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q6" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R6" s="20" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4392,7 +4611,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O7" s="20" t="n">
+      <c r="O7" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P7" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q7" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R7" s="20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5273,7 +5507,7 @@
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Holds every duty — inherently violates all 13 rules by design.</t>
+          <t>Holds every duty — inherently violates all 16 rules by design.</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -5871,7 +6105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5888,7 +6122,10 @@
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="6" customWidth="1" min="13" max="13"/>
     <col width="6" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5971,6 +6208,21 @@
       </c>
       <c r="O2" s="21" t="inlineStr">
         <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="P2" s="21" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="Q2" s="21" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="R2" s="21" t="inlineStr">
+        <is>
           <t># Conflicts</t>
         </is>
       </c>
@@ -6046,7 +6298,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O3" s="37" t="n">
+      <c r="O3" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P3" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q3" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R3" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6121,7 +6388,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O4" s="37" t="n">
+      <c r="O4" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P4" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q4" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R4" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6196,7 +6478,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O5" s="37" t="n">
+      <c r="O5" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P5" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q5" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R5" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6271,7 +6568,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O6" s="37" t="n">
+      <c r="O6" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P6" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q6" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R6" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6346,7 +6658,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O7" s="37" t="n">
+      <c r="O7" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P7" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q7" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R7" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6421,7 +6748,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O8" s="37" t="n">
+      <c r="O8" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P8" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q8" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R8" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6496,7 +6838,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O9" s="37" t="n">
+      <c r="O9" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P9" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q9" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R9" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6571,7 +6928,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O10" s="37" t="n">
+      <c r="O10" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P10" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q10" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R10" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6646,7 +7018,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O11" s="37" t="n">
+      <c r="O11" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P11" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q11" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R11" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6721,7 +7108,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O12" s="37" t="n">
+      <c r="O12" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P12" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q12" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R12" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6796,7 +7198,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O13" s="37" t="n">
+      <c r="O13" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P13" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q13" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R13" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6871,7 +7288,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O14" s="37" t="n">
+      <c r="O14" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P14" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q14" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R14" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6946,7 +7378,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O15" s="37" t="n">
+      <c r="O15" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P15" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q15" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R15" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7021,7 +7468,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O16" s="37" t="n">
+      <c r="O16" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P16" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q16" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R16" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7096,7 +7558,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O17" s="37" t="n">
+      <c r="O17" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P17" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q17" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R17" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7171,7 +7648,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O18" s="37" t="n">
+      <c r="O18" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P18" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q18" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R18" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7246,7 +7738,22 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O19" s="37" t="n">
+      <c r="O19" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="P19" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="Q19" s="25" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="R19" s="37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7321,7 +7828,22 @@
           <t>▲</t>
         </is>
       </c>
-      <c r="O20" s="24" t="inlineStr">
+      <c r="O20" s="23" t="inlineStr">
+        <is>
+          <t>▲</t>
+        </is>
+      </c>
+      <c r="P20" s="23" t="inlineStr">
+        <is>
+          <t>▲</t>
+        </is>
+      </c>
+      <c r="Q20" s="23" t="inlineStr">
+        <is>
+          <t>▲</t>
+        </is>
+      </c>
+      <c r="R20" s="24" t="inlineStr">
         <is>
           <t>ALL (▲)</t>
         </is>
@@ -7339,7 +7861,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A22:O24"/>
+    <mergeCell ref="A22:R24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>